<commit_message>
clarify optional XMLTV template fields
</commit_message>
<xml_diff>
--- a/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
+++ b/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="R5144e85ec39c46d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rc4b630c6dc074c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="R1ccb256738574115"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="R242c42e0b20e4e00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="Rdd0711050e944b25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R21bb06a781754b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="R5469e0728abb425d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rd8c75160832b4590"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -560,55 +560,55 @@
         <x:v>Program Title</x:v>
       </x:c>
       <x:c r="E4" s="14" t="str">
-        <x:v>Duration (Optional)</x:v>
+        <x:v>Duration (Conditional)</x:v>
       </x:c>
       <x:c r="F4" s="14" t="str">
         <x:v>Parental Rating</x:v>
       </x:c>
       <x:c r="G4" s="14" t="str">
-        <x:v>Program Description</x:v>
+        <x:v>Program Description (Conditional)</x:v>
       </x:c>
       <x:c r="H4" s="14" t="str">
-        <x:v>Original Title</x:v>
+        <x:v>Original Title (Optional)</x:v>
       </x:c>
       <x:c r="I4" s="14" t="str">
-        <x:v>Cast</x:v>
+        <x:v>Cast (Optional)</x:v>
       </x:c>
       <x:c r="J4" s="14" t="str">
-        <x:v>Season Number</x:v>
+        <x:v>Season Number (Optional)</x:v>
       </x:c>
       <x:c r="K4" s="14" t="str">
-        <x:v>Episode Number</x:v>
+        <x:v>Episode Number (Optional)</x:v>
       </x:c>
       <x:c r="L4" s="14" t="str">
-        <x:v>Original Episode Title</x:v>
+        <x:v>Original Episode Title (Optional)</x:v>
       </x:c>
       <x:c r="M4" s="14" t="str">
-        <x:v>Episode Description</x:v>
+        <x:v>Episode Description (Conditional)</x:v>
       </x:c>
       <x:c r="N4" s="14" t="str">
         <x:v>Genre</x:v>
       </x:c>
       <x:c r="O4" s="14" t="str">
-        <x:v>Country of Production</x:v>
+        <x:v>Country of Production (Optional)</x:v>
       </x:c>
       <x:c r="P4" s="14" t="str">
-        <x:v>Production Year</x:v>
+        <x:v>Production Year (Optional)</x:v>
       </x:c>
       <x:c r="Q4" s="14" t="str">
-        <x:v>Premiere</x:v>
+        <x:v>Premiere (Optional)</x:v>
       </x:c>
       <x:c r="R4" s="14" t="str">
-        <x:v>Live</x:v>
+        <x:v>Live (Optional)</x:v>
       </x:c>
       <x:c r="S4" s="14" t="str">
-        <x:v>New</x:v>
+        <x:v>New (Optional)</x:v>
       </x:c>
       <x:c r="T4" s="14" t="str">
         <x:v>Asset ID</x:v>
       </x:c>
       <x:c r="U4" s="14" t="str">
-        <x:v>Original Air Date</x:v>
+        <x:v>Original Air Date (Optional)</x:v>
       </x:c>
       <x:c r="V4" s="14" t="str">
         <x:v>Icon URL (Optional)</x:v>
@@ -623,7 +623,7 @@
         <x:v>Keywords (Optional)</x:v>
       </x:c>
       <x:c r="Z4" s="14" t="str">
-        <x:v>Previously Shown</x:v>
+        <x:v>Previously Shown (Optional)</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -14878,7 +14878,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="53" t="str">
-        <x:v>Duration (Optional)</x:v>
+        <x:v>Duration (Conditional)</x:v>
       </x:c>
       <x:c r="B9" s="53" t="str">
         <x:v>Programme duration. Required on the final row.</x:v>
@@ -14912,7 +14912,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="53" t="str">
-        <x:v>Program Description</x:v>
+        <x:v>Program Description (Conditional)</x:v>
       </x:c>
       <x:c r="B11" s="53" t="str">
         <x:v>Programme-level synopsis; fallback when episode description is blank.</x:v>
@@ -14929,7 +14929,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="53" t="str">
-        <x:v>Original Title</x:v>
+        <x:v>Original Title (Optional)</x:v>
       </x:c>
       <x:c r="B12" s="53" t="str">
         <x:v>Title in the original language.</x:v>
@@ -14946,7 +14946,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="53" t="str">
-        <x:v>Cast</x:v>
+        <x:v>Cast (Optional)</x:v>
       </x:c>
       <x:c r="B13" s="53" t="str">
         <x:v>Cast names separated by semicolons.</x:v>
@@ -14963,7 +14963,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="53" t="str">
-        <x:v>Season Number</x:v>
+        <x:v>Season Number (Optional)</x:v>
       </x:c>
       <x:c r="B14" s="53" t="str">
         <x:v>Season number for episodic content.</x:v>
@@ -14980,7 +14980,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="53" t="str">
-        <x:v>Episode Number</x:v>
+        <x:v>Episode Number (Optional)</x:v>
       </x:c>
       <x:c r="B15" s="53" t="str">
         <x:v>Episode number for episodic content.</x:v>
@@ -14997,7 +14997,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="53" t="str">
-        <x:v>Original Episode Title</x:v>
+        <x:v>Original Episode Title (Optional)</x:v>
       </x:c>
       <x:c r="B16" s="53" t="str">
         <x:v>Episode title.</x:v>
@@ -15014,7 +15014,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="53" t="str">
-        <x:v>Episode Description</x:v>
+        <x:v>Episode Description (Conditional)</x:v>
       </x:c>
       <x:c r="B17" s="53" t="str">
         <x:v>Episode synopsis; preferred XMLTV description.</x:v>
@@ -15048,7 +15048,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="53" t="str">
-        <x:v>Country of Production</x:v>
+        <x:v>Country of Production (Optional)</x:v>
       </x:c>
       <x:c r="B19" s="53" t="str">
         <x:v>Country where the content was produced.</x:v>
@@ -15065,7 +15065,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="53" t="str">
-        <x:v>Production Year</x:v>
+        <x:v>Production Year (Optional)</x:v>
       </x:c>
       <x:c r="B20" s="53" t="str">
         <x:v>Production year for internal metadata.</x:v>
@@ -15082,7 +15082,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="53" t="str">
-        <x:v>Premiere</x:v>
+        <x:v>Premiere (Optional)</x:v>
       </x:c>
       <x:c r="B21" s="53" t="str">
         <x:v>Indicates a premiere.</x:v>
@@ -15099,7 +15099,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="53" t="str">
-        <x:v>Live</x:v>
+        <x:v>Live (Optional)</x:v>
       </x:c>
       <x:c r="B22" s="53" t="str">
         <x:v>Indicates this specific airing is live.</x:v>
@@ -15116,7 +15116,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="53" t="str">
-        <x:v>New</x:v>
+        <x:v>New (Optional)</x:v>
       </x:c>
       <x:c r="B23" s="53" t="str">
         <x:v>Indicates a new episode or programme.</x:v>
@@ -15150,7 +15150,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="53" t="str">
-        <x:v>Original Air Date</x:v>
+        <x:v>Original Air Date (Optional)</x:v>
       </x:c>
       <x:c r="B25" s="53" t="str">
         <x:v>Original release or air date.</x:v>
@@ -15235,7 +15235,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="54" t="str">
-        <x:v>Previously Shown</x:v>
+        <x:v>Previously Shown (Optional)</x:v>
       </x:c>
       <x:c r="B30" s="54" t="str">
         <x:v>Indicates a repeat or previously aired programme.</x:v>
@@ -15319,55 +15319,55 @@
         <x:v>Program Title</x:v>
       </x:c>
       <x:c r="E4" s="14" t="str">
-        <x:v>Duration (Optional)</x:v>
+        <x:v>Duration (Conditional)</x:v>
       </x:c>
       <x:c r="F4" s="14" t="str">
         <x:v>Parental Rating</x:v>
       </x:c>
       <x:c r="G4" s="14" t="str">
-        <x:v>Program Description</x:v>
+        <x:v>Program Description (Conditional)</x:v>
       </x:c>
       <x:c r="H4" s="14" t="str">
-        <x:v>Original Title</x:v>
+        <x:v>Original Title (Optional)</x:v>
       </x:c>
       <x:c r="I4" s="14" t="str">
-        <x:v>Cast</x:v>
+        <x:v>Cast (Optional)</x:v>
       </x:c>
       <x:c r="J4" s="14" t="str">
-        <x:v>Season Number</x:v>
+        <x:v>Season Number (Optional)</x:v>
       </x:c>
       <x:c r="K4" s="14" t="str">
-        <x:v>Episode Number</x:v>
+        <x:v>Episode Number (Optional)</x:v>
       </x:c>
       <x:c r="L4" s="14" t="str">
-        <x:v>Original Episode Title</x:v>
+        <x:v>Original Episode Title (Optional)</x:v>
       </x:c>
       <x:c r="M4" s="14" t="str">
-        <x:v>Episode Description</x:v>
+        <x:v>Episode Description (Conditional)</x:v>
       </x:c>
       <x:c r="N4" s="14" t="str">
         <x:v>Genre</x:v>
       </x:c>
       <x:c r="O4" s="14" t="str">
-        <x:v>Country of Production</x:v>
+        <x:v>Country of Production (Optional)</x:v>
       </x:c>
       <x:c r="P4" s="14" t="str">
-        <x:v>Production Year</x:v>
+        <x:v>Production Year (Optional)</x:v>
       </x:c>
       <x:c r="Q4" s="14" t="str">
-        <x:v>Premiere</x:v>
+        <x:v>Premiere (Optional)</x:v>
       </x:c>
       <x:c r="R4" s="14" t="str">
-        <x:v>Live</x:v>
+        <x:v>Live (Optional)</x:v>
       </x:c>
       <x:c r="S4" s="14" t="str">
-        <x:v>New</x:v>
+        <x:v>New (Optional)</x:v>
       </x:c>
       <x:c r="T4" s="14" t="str">
         <x:v>Asset ID</x:v>
       </x:c>
       <x:c r="U4" s="14" t="str">
-        <x:v>Original Air Date</x:v>
+        <x:v>Original Air Date (Optional)</x:v>
       </x:c>
       <x:c r="V4" s="14" t="str">
         <x:v>Icon URL (Optional)</x:v>
@@ -15382,7 +15382,7 @@
         <x:v>Keywords (Optional)</x:v>
       </x:c>
       <x:c r="Z4" s="14" t="str">
-        <x:v>Previously Shown</x:v>
+        <x:v>Previously Shown (Optional)</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>

<commit_message>
generate XMLTV asset IDs automatically
</commit_message>
<xml_diff>
--- a/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
+++ b/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="Rdd0711050e944b25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R21bb06a781754b7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="R5469e0728abb425d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rd8c75160832b4590"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="Re1b3cb84639e45ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R99f943d54d3b4e5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="Re05237d4f37f4b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rfd09b92c84e44f3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -605,7 +605,7 @@
         <x:v>New (Optional)</x:v>
       </x:c>
       <x:c r="T4" s="14" t="str">
-        <x:v>Asset ID</x:v>
+        <x:v>Asset ID (Optional)</x:v>
       </x:c>
       <x:c r="U4" s="14" t="str">
         <x:v>Original Air Date (Optional)</x:v>
@@ -14698,7 +14698,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="40" t="str">
-        <x:v>Complete all required fields: Air Date, Start Time, Program Title, Description, Genre, Parental Rating, and Asset ID.</x:v>
+        <x:v>Complete all required fields: Air Date, Start Time, Program Title, Description, Genre, and Parental Rating.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -14714,7 +14714,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>Use a unique and stable Asset ID for every video asset.</x:v>
+        <x:v>Asset ID is optional. Leave it blank to let Broadcast Tool Pro generate it automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -15132,20 +15132,20 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="52" t="str">
-        <x:v>Asset ID</x:v>
-      </x:c>
-      <x:c r="B24" s="52" t="str">
-        <x:v>Unique video asset identifier.</x:v>
-      </x:c>
-      <x:c r="C24" s="52" t="str">
+      <x:c r="A24" s="53" t="str">
+        <x:v>Asset ID (Optional)</x:v>
+      </x:c>
+      <x:c r="B24" s="53" t="str">
+        <x:v>Unique video asset identifier. Generated automatically when blank.</x:v>
+      </x:c>
+      <x:c r="C24" s="53" t="str">
         <x:v>Text</x:v>
       </x:c>
-      <x:c r="D24" s="52" t="str">
+      <x:c r="D24" s="53" t="str">
         <x:v>morning-news-s01e01</x:v>
       </x:c>
-      <x:c r="E24" s="52" t="str">
-        <x:v>Required</x:v>
+      <x:c r="E24" s="53" t="str">
+        <x:v>Optional</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -15364,7 +15364,7 @@
         <x:v>New (Optional)</x:v>
       </x:c>
       <x:c r="T4" s="14" t="str">
-        <x:v>Asset ID</x:v>
+        <x:v>Asset ID (Optional)</x:v>
       </x:c>
       <x:c r="U4" s="14" t="str">
         <x:v>Original Air Date (Optional)</x:v>

</xml_diff>

<commit_message>
enforce ISO date formatting in XMLTV template
</commit_message>
<xml_diff>
--- a/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
+++ b/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="Re1b3cb84639e45ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R99f943d54d3b4e5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="Re05237d4f37f4b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rfd09b92c84e44f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="R445257ac5f204b76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rd530aae319104853"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="R1a072fed44c14b94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rc597ba3d54894360"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14632,7 +14632,15 @@
     <x:mergeCell ref="B2:Z2"/>
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
-  <x:dataValidations count="3">
+  <x:dataValidations count="5">
+    <x:dataValidation type="date" operator="between" sqref="B5:B504">
+      <x:formula1>36526</x:formula1>
+      <x:formula2>73415</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="date" operator="between" sqref="U5:U504">
+      <x:formula1>36526</x:formula1>
+      <x:formula2>73415</x:formula2>
+    </x:dataValidation>
     <x:dataValidation type="list" sqref="Q5:S504">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>

</xml_diff>

<commit_message>
Apply official Broadcast Tool Pro branding
</commit_message>
<xml_diff>
--- a/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
+++ b/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="R445257ac5f204b76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rd530aae319104853"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="R1a072fed44c14b94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rc597ba3d54894360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="Re3238f01fdd24b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R9bad73d105094036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="Re7bceb01e78c4f19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rfb71bbb2f44a461d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -310,6 +310,134 @@
 </x:styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2714625" cy="600075"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="f2e16fed-bfa5-4adc-9552-9e60a722f84d"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6eb52436c21a4775"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2714625" cy="600075"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="9449fec1-d45b-4ee6-8b72-9b5c7f981209"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re831f434ce6e44dc"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2714625" cy="600075"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="b6aea613-91d3-4832-a26d-98f5c1c6c04e"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb6ec04f0ad0444fa"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2714625" cy="600075"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="956ebe01-ee7c-40b8-a439-ecd15d17c95c"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R33d579452ae046af"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
@@ -14652,6 +14780,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b1db5cfc8ab4ebe"/>
 </x:worksheet>
 </file>
 
@@ -14772,6 +14901,7 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb294ccea4ea644aa"/>
 </x:worksheet>
 </file>
 
@@ -15265,6 +15395,7 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3313cf19818459d"/>
 </x:worksheet>
 </file>
 
@@ -15554,5 +15685,6 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree6c117e9cc641c9"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine transparent brand layouts
</commit_message>
<xml_diff>
--- a/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
+++ b/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="Re3238f01fdd24b22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R9bad73d105094036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="Re7bceb01e78c4f19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rfb71bbb2f44a461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="R9cb508643cab48ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R554baad1f3f24a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="Rea22f976faac4790"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="R71f6e2dd27b7460c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -65,7 +65,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -102,8 +102,13 @@
         <x:fgColor rgb="FFDBEAFE"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="5">
+  <x:borders count="7">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -137,11 +142,33 @@
         <x:color rgb="FFD7E1EC"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7E1EC"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7E1EC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7E1EC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7E1EC"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7E1EC"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7E1EC"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="77">
+  <x:cellXfs count="81">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -303,6 +330,14 @@
     <x:xf numFmtId="202" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -315,20 +350,20 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>342900</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2714625" cy="600075"/>
+    <xdr:ext cx="514350" cy="485775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="f2e16fed-bfa5-4adc-9552-9e60a722f84d"/>
+        <xdr:cNvPr id="1" name="7b2b0dbd-6689-4fcd-8050-f8844ed910eb"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6eb52436c21a4775"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R56a1b7f8966245fb"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -349,18 +384,18 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>76200</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2714625" cy="600075"/>
+    <xdr:ext cx="514350" cy="485775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="9449fec1-d45b-4ee6-8b72-9b5c7f981209"/>
+        <xdr:cNvPr id="1" name="89efe932-c0c9-4679-bd71-0115b0d3537c"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re831f434ce6e44dc"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbfc78c9fe58c4d2d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -379,20 +414,20 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>685800</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2714625" cy="600075"/>
+    <xdr:ext cx="514350" cy="485775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="b6aea613-91d3-4832-a26d-98f5c1c6c04e"/>
+        <xdr:cNvPr id="1" name="59e5e7e8-7081-42c6-a107-ed91f3ceb0e2"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb6ec04f0ad0444fa"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1758dcf4f4784990"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -411,20 +446,20 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>342900</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2714625" cy="600075"/>
+    <xdr:ext cx="514350" cy="485775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="956ebe01-ee7c-40b8-a439-ecd15d17c95c"/>
+        <xdr:cNvPr id="1" name="b54c0c0c-c703-40d6-b87d-98ffd902dbb7"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R33d579452ae046af"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re44f762aa53d4bba"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -662,14 +697,13 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>B</x:v>
-      </x:c>
+      <x:c r="A1" s="79" t="str"/>
       <x:c r="B1" s="7" t="str">
         <x:v>Broadcast Tool Pro - XMLTV Programming Template</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="80"/>
       <x:c r="B2" s="10" t="str">
         <x:v>Enter one row per programme using the channel's local time zone.</x:v>
       </x:c>
@@ -14780,7 +14814,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b1db5cfc8ab4ebe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11fe917134e54f03"/>
 </x:worksheet>
 </file>
 
@@ -14794,14 +14828,13 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>B</x:v>
-      </x:c>
+      <x:c r="A1" s="79" t="str"/>
       <x:c r="B1" s="7" t="str">
         <x:v>How to Use This Template</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="80"/>
       <x:c r="B2" s="10" t="str">
         <x:v>Keep the worksheet name and column headers unchanged.</x:v>
       </x:c>
@@ -14901,7 +14934,7 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb294ccea4ea644aa"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce9d637f8be844fd"/>
 </x:worksheet>
 </file>
 
@@ -14917,14 +14950,13 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>B</x:v>
-      </x:c>
+      <x:c r="A1" s="79" t="str"/>
       <x:c r="B1" s="7" t="str">
         <x:v>XMLTV Field Reference</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="80"/>
       <x:c r="B2" s="10" t="str">
         <x:v>Required fields are highlighted in blue; optional fields are shown in gray.</x:v>
       </x:c>
@@ -15395,7 +15427,7 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3313cf19818459d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd67c297fb7264f93"/>
 </x:worksheet>
 </file>
 
@@ -15432,14 +15464,13 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>B</x:v>
-      </x:c>
+      <x:c r="A1" s="79" t="str"/>
       <x:c r="B1" s="7" t="str">
         <x:v>Completed Example - Do Not Upload This Sheet</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="80"/>
       <x:c r="B2" s="10" t="str">
         <x:v>Copy the field patterns, then enter your real schedule on Programming.</x:v>
       </x:c>
@@ -15685,6 +15716,6 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree6c117e9cc641c9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4125dabadd5a4cd9"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Enforce registered channel identity
</commit_message>
<xml_diff>
--- a/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
+++ b/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="R9cb508643cab48ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R554baad1f3f24a50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="Rea22f976faac4790"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="R71f6e2dd27b7460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="R1cdc47c3c3524ee5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R49b2429a79a44bac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="Rd5e688b0cb504e61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rdc752a4b3db842b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -65,7 +65,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -105,6 +105,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -168,7 +173,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="81">
+  <x:cellXfs count="82">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -338,6 +343,9 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -357,13 +365,13 @@
     <xdr:ext cx="514350" cy="485775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="7b2b0dbd-6689-4fcd-8050-f8844ed910eb"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R56a1b7f8966245fb"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R38fb1c1e3e5445fe"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -389,13 +397,13 @@
     <xdr:ext cx="514350" cy="485775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="89efe932-c0c9-4679-bd71-0115b0d3537c"/>
+        <xdr:cNvPr id="1" name="/xl/media/image2.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbfc78c9fe58c4d2d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rece1e598edcf4775"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -421,13 +429,13 @@
     <xdr:ext cx="514350" cy="485775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="59e5e7e8-7081-42c6-a107-ed91f3ceb0e2"/>
+        <xdr:cNvPr id="1" name="/xl/media/image3.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1758dcf4f4784990"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb178b4286bef44f9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -453,13 +461,13 @@
     <xdr:ext cx="514350" cy="485775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="b54c0c0c-c703-40d6-b87d-98ffd902dbb7"/>
+        <xdr:cNvPr id="1" name="/xl/media/image4.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re44f762aa53d4bba"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0b375202d2724a30"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -710,7 +718,7 @@
     </x:row>
     <x:row r="4" ht="44" customHeight="1">
       <x:c r="A4" s="14" t="str">
-        <x:v>Channel (Optional)</x:v>
+        <x:v>Channel</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
         <x:v>Air Date</x:v>
@@ -14814,7 +14822,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11fe917134e54f03"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb08a3c02a5014dea"/>
 </x:worksheet>
 </file>
 
@@ -14868,7 +14876,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="40" t="str">
-        <x:v>Complete all required fields: Air Date, Start Time, Program Title, Description, Genre, and Parental Rating.</x:v>
+        <x:v>Complete all required fields: Channel, Air Date, Start Time, Program Title, Description, Genre, and Parental Rating.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -14916,7 +14924,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B13" s="40" t="str">
-        <x:v>Save the workbook as .xlsx, upload it, and select the channel's IANA time zone.</x:v>
+        <x:v>Save the workbook as .xlsx and upload it under the selected registered channel.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -14934,7 +14942,7 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce9d637f8be844fd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca91a55421e44b3c"/>
 </x:worksheet>
 </file>
 
@@ -14979,20 +14987,20 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="51" t="str">
-        <x:v>Channel (Optional)</x:v>
-      </x:c>
-      <x:c r="B5" s="51" t="str">
-        <x:v>Channel name or ID.</x:v>
-      </x:c>
-      <x:c r="C5" s="51" t="str">
+      <x:c r="A5" s="81" t="str">
+        <x:v>Channel</x:v>
+      </x:c>
+      <x:c r="B5" s="81" t="str">
+        <x:v>Registered channel name. It must match the selected BTP channel on every programme row.</x:v>
+      </x:c>
+      <x:c r="C5" s="81" t="str">
         <x:v>Text</x:v>
       </x:c>
-      <x:c r="D5" s="51" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>Comercio TV</x:v>
       </x:c>
-      <x:c r="E5" s="51" t="str">
-        <x:v>Optional</x:v>
+      <x:c r="E5" s="81" t="str">
+        <x:v>Required</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -15427,7 +15435,7 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd67c297fb7264f93"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1de0c1f39cca4f64"/>
 </x:worksheet>
 </file>
 
@@ -15477,7 +15485,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="14" t="str">
-        <x:v>Channel (Optional)</x:v>
+        <x:v>Channel</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
         <x:v>Air Date</x:v>
@@ -15716,6 +15724,6 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4125dabadd5a4cd9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R483c02638b1f44ee"/>
 </x:worksheet>
 </file>
</xml_diff>